<commit_message>
feat: worked on colum selection
</commit_message>
<xml_diff>
--- a/artifacts/reports/lending_club_accepted_col_selection.xlsx
+++ b/artifacts/reports/lending_club_accepted_col_selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pragyan/Desktop/Projects/credit-risk-prediction-system/artifacts/reports/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{362C329D-1C28-7441-A066-312C428426E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B359ED1-AB15-AD4A-9F7A-A2D0D25C5B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{330B8E5A-0C55-B24A-B397-B8858ABF4B19}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="637" uniqueCount="471">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="645" uniqueCount="476">
   <si>
     <t>column</t>
   </si>
@@ -1449,6 +1449,21 @@
   <si>
     <t>recoveries is money collected after a loan has already been charged off (defaulted), typically via collection efforts.
 This is post default. So it's a leakage</t>
+  </si>
+  <si>
+    <t>This is post default. So it's a leakage</t>
+  </si>
+  <si>
+    <t>Every row has same value</t>
+  </si>
+  <si>
+    <t>This is post T0. So it's a leakage</t>
+  </si>
+  <si>
+    <t>Use fico_range_low</t>
+  </si>
+  <si>
+    <t>Use fico_range_high</t>
   </si>
 </sst>
 </file>
@@ -2016,13 +2031,13 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2031,13 +2046,13 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="35" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1"/>
@@ -2704,7 +2719,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="12" spans="1:8" s="6" customFormat="1" ht="187">
+    <row r="12" spans="1:8" s="6" customFormat="1" ht="170">
       <c r="A12" s="12">
         <v>10</v>
       </c>
@@ -3609,173 +3624,187 @@
         <v>470</v>
       </c>
     </row>
-    <row r="48" spans="1:8" ht="34">
-      <c r="A48" s="9">
+    <row r="48" spans="1:8" s="5" customFormat="1" ht="34">
+      <c r="A48" s="7">
         <v>46</v>
       </c>
-      <c r="B48" s="9" t="s">
+      <c r="B48" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="D48" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E48" s="9">
+      <c r="D48" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E48" s="7">
         <v>0</v>
       </c>
-      <c r="F48" s="9">
+      <c r="F48" s="7">
         <v>146222</v>
       </c>
-      <c r="G48" s="9" t="s">
+      <c r="G48" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="H48" s="9"/>
-    </row>
-    <row r="49" spans="1:8" ht="34">
-      <c r="A49" s="9">
+      <c r="H48" s="7" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8" s="5" customFormat="1" ht="34">
+      <c r="A49" s="7">
         <v>47</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B49" s="7" t="s">
         <v>146</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="D49" s="9" t="s">
+      <c r="D49" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E49" s="9">
+      <c r="E49" s="7">
         <v>0.11</v>
       </c>
-      <c r="F49" s="9">
+      <c r="F49" s="7">
         <v>136</v>
       </c>
-      <c r="G49" s="9" t="s">
+      <c r="G49" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="H49" s="9"/>
-    </row>
-    <row r="50" spans="1:8" ht="34">
-      <c r="A50" s="9">
+      <c r="H49" s="7" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8" s="5" customFormat="1" ht="34">
+      <c r="A50" s="7">
         <v>48</v>
       </c>
-      <c r="B50" s="9" t="s">
+      <c r="B50" s="7" t="s">
         <v>149</v>
       </c>
-      <c r="C50" s="9" t="s">
+      <c r="C50" s="7" t="s">
         <v>150</v>
       </c>
-      <c r="D50" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E50" s="9">
+      <c r="D50" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E50" s="7">
         <v>0</v>
       </c>
-      <c r="F50" s="9">
+      <c r="F50" s="7">
         <v>704467</v>
       </c>
-      <c r="G50" s="9" t="s">
+      <c r="G50" s="7" t="s">
         <v>151</v>
       </c>
-      <c r="H50" s="9"/>
-    </row>
-    <row r="51" spans="1:8" ht="34">
-      <c r="A51" s="9">
+      <c r="H50" s="7" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="51" spans="1:8" s="5" customFormat="1" ht="34">
+      <c r="A51" s="7">
         <v>49</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B51" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="7" t="s">
         <v>153</v>
       </c>
-      <c r="D51" s="9" t="s">
+      <c r="D51" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E51" s="9">
+      <c r="E51" s="7">
         <v>59.51</v>
       </c>
-      <c r="F51" s="9">
+      <c r="F51" s="7">
         <v>106</v>
       </c>
-      <c r="G51" s="9" t="s">
+      <c r="G51" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="H51" s="9"/>
-    </row>
-    <row r="52" spans="1:8" ht="34">
-      <c r="A52" s="9">
+      <c r="H51" s="7" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8" s="5" customFormat="1" ht="34">
+      <c r="A52" s="7">
         <v>50</v>
       </c>
-      <c r="B52" s="9" t="s">
+      <c r="B52" s="7" t="s">
         <v>155</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="D52" s="9" t="s">
+      <c r="D52" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="E52" s="9">
+      <c r="E52" s="7">
         <v>0</v>
       </c>
-      <c r="F52" s="9">
+      <c r="F52" s="7">
         <v>141</v>
       </c>
-      <c r="G52" s="9" t="s">
+      <c r="G52" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="H52" s="9"/>
-    </row>
-    <row r="53" spans="1:8" ht="34">
-      <c r="A53" s="9">
+      <c r="H52" s="7" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8" s="5" customFormat="1" ht="34">
+      <c r="A53" s="7">
         <v>51</v>
       </c>
-      <c r="B53" s="9" t="s">
+      <c r="B53" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="D53" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E53" s="9">
+      <c r="D53" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E53" s="7">
         <v>0</v>
       </c>
-      <c r="F53" s="9">
+      <c r="F53" s="7">
         <v>72</v>
       </c>
-      <c r="G53" s="9" t="s">
+      <c r="G53" s="7" t="s">
         <v>160</v>
       </c>
-      <c r="H53" s="9"/>
-    </row>
-    <row r="54" spans="1:8" ht="34">
-      <c r="A54" s="9">
+      <c r="H53" s="7" t="s">
+        <v>475</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8" s="5" customFormat="1" ht="34">
+      <c r="A54" s="7">
         <v>52</v>
       </c>
-      <c r="B54" s="9" t="s">
+      <c r="B54" s="7" t="s">
         <v>161</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D54" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E54" s="9">
+      <c r="D54" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E54" s="7">
         <v>0</v>
       </c>
-      <c r="F54" s="9">
+      <c r="F54" s="7">
         <v>71</v>
       </c>
-      <c r="G54" s="9" t="s">
+      <c r="G54" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="H54" s="9"/>
+      <c r="H54" s="7" t="s">
+        <v>474</v>
+      </c>
     </row>
     <row r="55" spans="1:8" ht="51">
       <c r="A55" s="9">
@@ -3825,29 +3854,31 @@
       </c>
       <c r="H56" s="9"/>
     </row>
-    <row r="57" spans="1:8" ht="51">
-      <c r="A57" s="9">
+    <row r="57" spans="1:8" s="5" customFormat="1" ht="51">
+      <c r="A57" s="7">
         <v>55</v>
       </c>
-      <c r="B57" s="9" t="s">
+      <c r="B57" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="C57" s="9" t="s">
+      <c r="C57" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="D57" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E57" s="9">
+      <c r="D57" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E57" s="7">
         <v>0</v>
       </c>
-      <c r="F57" s="9">
+      <c r="F57" s="7">
         <v>1</v>
       </c>
-      <c r="G57" s="9" t="s">
+      <c r="G57" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="H57" s="9"/>
+      <c r="H57" s="7" t="s">
+        <v>472</v>
+      </c>
     </row>
     <row r="58" spans="1:8" ht="51">
       <c r="A58" s="9">

</xml_diff>